<commit_message>
Auto update portfolio 2026-10-30 12:29 UTC
</commit_message>
<xml_diff>
--- a/data/MyPortfolio.xlsx
+++ b/data/MyPortfolio.xlsx
@@ -638,41 +638,41 @@
         <v>1741.62</v>
       </c>
       <c r="J2" s="11" t="n">
-        <v>16588000</v>
+        <v>17668000</v>
       </c>
       <c r="K2" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L2" s="11" t="n">
-        <v>16751000</v>
+        <v>17868500</v>
       </c>
       <c r="M2" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>-0.009730762342546714</v>
+        <v>-0.01122086353079441</v>
       </c>
       <c r="O2" s="12" t="n">
         <v>-0.007968740209955527</v>
       </c>
       <c r="P2" s="12" t="n">
-        <v>-0.294626767050114</v>
+        <v>-0.24870181578499</v>
       </c>
       <c r="Q2" s="12" t="n">
-        <v>-0.3898209364556551</v>
+        <v>-0.3500938211537562</v>
       </c>
       <c r="R2" s="12" t="n">
-        <v>-0.7587678226781063</v>
+        <v>-0.7430618453747753</v>
       </c>
       <c r="S2" s="12" t="n">
         <v>-0.02402367062858168</v>
       </c>
       <c r="T2" s="6">
-        <f>(-0.7587678226781063 - 0.04) / (STDEVP(N2:N205) * SQRT(252))</f>
+        <f>(-0.7430618453747753 - 0.04) / (STDEVP(N2:N205) * SQRT(252))</f>
         <v/>
       </c>
       <c r="U2" s="12" t="n">
-        <v>-0.7844521941143038</v>
+        <v>-0.7704184570539858</v>
       </c>
     </row>
     <row r="3">
@@ -706,25 +706,25 @@
         <v>1755.61</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>16751000</v>
+        <v>17868500</v>
       </c>
       <c r="K3" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>18240000</v>
+        <v>19915000</v>
       </c>
       <c r="M3" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>-0.08163377192982456</v>
+        <v>-0.1027617373838815</v>
       </c>
       <c r="O3" s="12" t="n">
         <v>-0.006249115557694029</v>
       </c>
       <c r="P3" s="12" t="n">
-        <v>-0.2876955012573222</v>
+        <v>-0.2401759336288257</v>
       </c>
       <c r="Q3" s="13" t="n"/>
       <c r="R3" s="13" t="n"/>
@@ -763,25 +763,25 @@
         <v>1766.65</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>18240000</v>
+        <v>19915000</v>
       </c>
       <c r="K4" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>18971000</v>
+        <v>20648500</v>
       </c>
       <c r="M4" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>-0.03853249696905803</v>
+        <v>-0.03552316148872799</v>
       </c>
       <c r="O4" s="12" t="n">
         <v>0.002713026500252624</v>
       </c>
       <c r="P4" s="12" t="n">
-        <v>-0.2243786008556837</v>
+        <v>-0.1531524032917181</v>
       </c>
       <c r="Q4" s="13" t="n"/>
       <c r="R4" s="13" t="n"/>
@@ -820,25 +820,25 @@
         <v>1761.87</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>18971000</v>
+        <v>20648500</v>
       </c>
       <c r="K5" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>19216000</v>
+        <v>20906000</v>
       </c>
       <c r="M5" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>-0.01274979184013322</v>
+        <v>-0.01231703817086004</v>
       </c>
       <c r="O5" s="12" t="n">
         <v>-0.0009526239686995508</v>
       </c>
       <c r="P5" s="12" t="n">
-        <v>-0.1932942125456785</v>
+        <v>-0.1219617072241547</v>
       </c>
       <c r="Q5" s="13" t="n"/>
       <c r="R5" s="13" t="n"/>
@@ -877,25 +877,25 @@
         <v>1763.55</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>19216000</v>
+        <v>20906000</v>
       </c>
       <c r="K6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>19718000</v>
+        <v>21428000</v>
       </c>
       <c r="M6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>-0.02545897149812354</v>
+        <v>-0.02436064961732313</v>
       </c>
       <c r="O6" s="12" t="n">
         <v>-0.005974692106079038</v>
       </c>
       <c r="P6" s="12" t="n">
-        <v>-0.1828760523049791</v>
+        <v>-0.1110120081956645</v>
       </c>
       <c r="Q6" s="13" t="n"/>
       <c r="R6" s="13" t="n"/>
@@ -934,25 +934,25 @@
         <v>1774.15</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>19718000</v>
+        <v>21428000</v>
       </c>
       <c r="K7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>20021000</v>
+        <v>21728500</v>
       </c>
       <c r="M7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>-0.01513410918535538</v>
+        <v>-0.0138297627539867</v>
       </c>
       <c r="O7" s="12" t="n">
         <v>0.007679069424012974</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>-0.1615294545873011</v>
+        <v>-0.08881494841752124</v>
       </c>
       <c r="Q7" s="13" t="n"/>
       <c r="R7" s="13" t="n"/>
@@ -991,25 +991,25 @@
         <v>1760.63</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>20021000</v>
+        <v>21728500</v>
       </c>
       <c r="K8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="11" t="n">
-        <v>20002000</v>
+        <v>21722000</v>
       </c>
       <c r="M8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>0.0009499050094990501</v>
+        <v>0.0002992357978086733</v>
       </c>
       <c r="O8" s="12" t="n">
         <v>0.01263034388354312</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>-0.1486449543712524</v>
+        <v>-0.0760367559590307</v>
       </c>
       <c r="Q8" s="13" t="n"/>
       <c r="R8" s="13" t="n"/>
@@ -1048,25 +1048,25 @@
         <v>1738.67</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>20002000</v>
+        <v>21722000</v>
       </c>
       <c r="K9" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>19935000</v>
+        <v>21632500</v>
       </c>
       <c r="M9" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>0.003360922999749185</v>
+        <v>0.004137293424245926</v>
       </c>
       <c r="O9" s="12" t="n">
         <v>0.02760096219200103</v>
       </c>
       <c r="P9" s="12" t="n">
-        <v>-0.1494528933286943</v>
+        <v>-0.07631315612868195</v>
       </c>
       <c r="Q9" s="13" t="n"/>
       <c r="R9" s="13" t="n"/>
@@ -1105,25 +1105,25 @@
         <v>1691.97</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>19935000</v>
+        <v>21632500</v>
       </c>
       <c r="K10" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="11" t="n">
-        <v>19491000</v>
+        <v>21153500</v>
       </c>
       <c r="M10" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>0.02277974449746037</v>
+        <v>0.02264400690193112</v>
       </c>
       <c r="O10" s="12" t="n">
         <v>0.001260474364436881</v>
       </c>
       <c r="P10" s="12" t="n">
-        <v>-0.1523019412312528</v>
+        <v>-0.08011897384926392</v>
       </c>
       <c r="Q10" s="13" t="n"/>
       <c r="R10" s="13" t="n"/>
@@ -1162,7 +1162,7 @@
         <v>1689.84</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>19491000</v>
+        <v>21153500</v>
       </c>
       <c r="K11" s="11" t="n">
         <v>0</v>
@@ -1174,13 +1174,13 @@
         <v>0</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>-0.03145497912939774</v>
+        <v>0.05115782150665871</v>
       </c>
       <c r="O11" s="12" t="n">
         <v>-0.00942019215550649</v>
       </c>
       <c r="P11" s="12" t="n">
-        <v>-0.1711821989735817</v>
+        <v>-0.1004875401974069</v>
       </c>
       <c r="Q11" s="13" t="n"/>
       <c r="R11" s="13" t="n"/>

</xml_diff>